<commit_message>
tidied up the de trial docs
</commit_message>
<xml_diff>
--- a/DE-trial-results/DE Trial — Scorecard (Responses).xlsx
+++ b/DE-trial-results/DE Trial — Scorecard (Responses).xlsx
@@ -957,6 +957,12 @@
       <c r="E9" s="8" t="s">
         <v>47</v>
       </c>
+      <c r="F9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="H9" s="8" t="s">
         <v>20</v>
       </c>

</xml_diff>